<commit_message>
fix: corrigir formula do IAD - weight somado a fracao, nao no denominador
</commit_message>
<xml_diff>
--- a/docs/validacao/Folha_Calculo_IAD_Pokemon.xlsx
+++ b/docs/validacao/Folha_Calculo_IAD_Pokemon.xlsx
@@ -559,11 +559,11 @@
         <v>0.75</v>
       </c>
       <c r="L2" s="2">
-        <f t="shared" ref="L2:L11" si="3">ROUND((((B2*J2)+(C2*E2))/(((D2+1)*(F2+1))+G2))*K2,2)</f>
-        <v>4.39</v>
+        <f t="shared" ref="L2:L11" si="3">ROUND((((B2*J2)+(C2*E2))/((D2+1)*(F2+1))+G2)*K2,2)</f>
+        <v>56.90</v>
       </c>
       <c r="M2" s="2">
-        <v>4.39</v>
+        <v>56.90</v>
       </c>
       <c r="N2" s="2" t="str">
         <f t="shared" ref="N2:N11" si="4">IF(M2="","",IF(ABS(L2-M2)&lt;0.005,"OK","DIFF"))</f>
@@ -606,10 +606,10 @@
       </c>
       <c r="L3" s="2">
         <f t="shared" si="3"/>
-        <v>12.68</v>
+        <v>130.93</v>
       </c>
       <c r="M3" s="3">
-        <v>12.68</v>
+        <v>130.93</v>
       </c>
       <c r="N3" s="2" t="str">
         <f t="shared" si="4"/>
@@ -654,10 +654,10 @@
       </c>
       <c r="L4" s="2">
         <f t="shared" si="3"/>
-        <v>5.51</v>
+        <v>1230.76</v>
       </c>
       <c r="M4" s="3">
-        <v>5.51</v>
+        <v>1230.76</v>
       </c>
       <c r="N4" s="2" t="str">
         <f t="shared" si="4"/>
@@ -700,10 +700,10 @@
       </c>
       <c r="L5" s="2">
         <f t="shared" si="3"/>
-        <v>26.64</v>
+        <v>115.44</v>
       </c>
       <c r="M5" s="3">
-        <v>26.64</v>
+        <v>115.44</v>
       </c>
       <c r="N5" s="2" t="str">
         <f t="shared" si="4"/>
@@ -748,10 +748,10 @@
       </c>
       <c r="L6" s="2">
         <f t="shared" si="3"/>
-        <v>0.21</v>
+        <v>2100.24</v>
       </c>
       <c r="M6" s="3">
-        <v>0.21</v>
+        <v>2100.24</v>
       </c>
       <c r="N6" s="2" t="str">
         <f t="shared" si="4"/>
@@ -794,10 +794,10 @@
       </c>
       <c r="L7" s="2">
         <f t="shared" si="3"/>
-        <v>12.06</v>
+        <v>80.91</v>
       </c>
       <c r="M7" s="3">
-        <v>12.06</v>
+        <v>80.91</v>
       </c>
       <c r="N7" s="2" t="str">
         <f t="shared" si="4"/>
@@ -840,10 +840,10 @@
       </c>
       <c r="L8" s="2">
         <f t="shared" si="3"/>
-        <v>0.65</v>
+        <v>4602.71</v>
       </c>
       <c r="M8" s="3">
-        <v>0.65</v>
+        <v>4602.71</v>
       </c>
       <c r="N8" s="2" t="str">
         <f t="shared" si="4"/>
@@ -888,10 +888,10 @@
       </c>
       <c r="L9" s="2">
         <f t="shared" si="3"/>
-        <v>2.83</v>
+        <v>2105.51</v>
       </c>
       <c r="M9" s="3">
-        <v>2.83</v>
+        <v>2105.51</v>
       </c>
       <c r="N9" s="2" t="str">
         <f t="shared" si="4"/>
@@ -934,10 +934,10 @@
       </c>
       <c r="L10" s="2">
         <f t="shared" si="3"/>
-        <v>4.77</v>
+        <v>1227.82</v>
       </c>
       <c r="M10" s="3">
-        <v>4.77</v>
+        <v>1227.82</v>
       </c>
       <c r="N10" s="2" t="str">
         <f t="shared" si="4"/>
@@ -982,10 +982,10 @@
       </c>
       <c r="L11" s="2">
         <f t="shared" si="3"/>
-        <v>2.18</v>
+        <v>507.62</v>
       </c>
       <c r="M11" s="3">
-        <v>2.18</v>
+        <v>507.62</v>
       </c>
       <c r="N11" s="2" t="str">
         <f t="shared" si="4"/>

</xml_diff>